<commit_message>
Add cleaned and split data for TCN project
</commit_message>
<xml_diff>
--- a/labeled/june/inspection/sip_volume_distribution_after_augmentation.xlsx
+++ b/labeled/june/inspection/sip_volume_distribution_after_augmentation.xlsx
@@ -624,7 +624,7 @@
         <v>67.5</v>
       </c>
       <c r="C15" t="n">
-        <v>72</v>
+        <v>84</v>
       </c>
     </row>
     <row r="16">
@@ -637,7 +637,7 @@
         <v>72.5</v>
       </c>
       <c r="C16" t="n">
-        <v>72</v>
+        <v>84</v>
       </c>
     </row>
     <row r="17">
@@ -676,7 +676,7 @@
         <v>87.5</v>
       </c>
       <c r="C19" t="n">
-        <v>62</v>
+        <v>60</v>
       </c>
     </row>
     <row r="20">
@@ -689,7 +689,7 @@
         <v>92.5</v>
       </c>
       <c r="C20" t="n">
-        <v>93</v>
+        <v>69</v>
       </c>
     </row>
     <row r="21">
@@ -767,7 +767,7 @@
         <v>122.5</v>
       </c>
       <c r="C26" t="n">
-        <v>7</v>
+        <v>37</v>
       </c>
     </row>
     <row r="27">
@@ -780,7 +780,7 @@
         <v>127.5</v>
       </c>
       <c r="C27" t="n">
-        <v>7</v>
+        <v>37</v>
       </c>
     </row>
     <row r="28">
@@ -793,7 +793,7 @@
         <v>132.5</v>
       </c>
       <c r="C28" t="n">
-        <v>7</v>
+        <v>37</v>
       </c>
     </row>
     <row r="29">
@@ -819,7 +819,7 @@
         <v>142.5</v>
       </c>
       <c r="C30" t="n">
-        <v>7</v>
+        <v>32</v>
       </c>
     </row>
     <row r="31">
@@ -871,7 +871,7 @@
         <v>162.5</v>
       </c>
       <c r="C34" t="n">
-        <v>7</v>
+        <v>32</v>
       </c>
     </row>
   </sheetData>

</xml_diff>